<commit_message>
Fix unconfirmed 2019 margin and rounded text, add SQL queries, sensitivity table, loss-share CSV
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01T57CWqisSdhbNGN4esb2BE
</commit_message>
<xml_diff>
--- a/data/Canadian_Restaurant_Benchmark.xlsx
+++ b/data/Canadian_Restaurant_Benchmark.xlsx
@@ -270,13 +270,13 @@
     <t xml:space="preserve">What the data says</t>
   </si>
   <si>
-    <t xml:space="preserve">In 2020 full-service restaurants fell to a 0.3% margin while limited-service (take-out and counter) places earned 5.3%. Limited-service (counter and take-out style) places held up far better than full-service.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Industry margins stay thin (3% to 4%) in every year, so small cost improvements matter.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Cost of goods sold is about 35% to 36% and wages about 32% to 34% of expenses every year.</t>
+    <t xml:space="preserve">In 2020 full-service restaurants fell to a 0.3% operating margin while limited-service (take-out and counter) places earned 5.3%, as published in the 2020 release (a later release shows 0.5% for full-service 2020, so 2020 was revised). Revenue columns for full-service and limited-service do not add up to the total because drinking places and other food services are not shown.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Industry operating margins stay thin in every year (2.9% to 4.3%), so small cost improvements matter.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cost of goods sold is 34.8% to 35.9% and wages 32.0% to 33.6% of operating expenses in the years reported.</t>
   </si>
   <si>
     <t xml:space="preserve">Workforce (Statistics Canada, 2025): salaries, wages and commissions rose 22.2% from 2019 to 2023; job vacancy rate peaked at 13.4% in Q3 2021, then 10.2% in 2022 and 7.1% in 2023.</t>
@@ -2953,9 +2953,7 @@
       <c r="G5" s="21" t="n">
         <v>0.03</v>
       </c>
-      <c r="H5" s="21" t="n">
-        <v>0.039</v>
-      </c>
+      <c r="H5" s="21"/>
       <c r="I5" s="21" t="n">
         <v>0.359</v>
       </c>

</xml_diff>

<commit_message>
Add conservative case, number checks, CI and a clean install
- requirements.txt; run_queries.py no longer crashes without tabulate
- conservative scenario (published cost lines only), per-1% lever table, waste-share range
- checks.py recomputes every headline number and compares README, dashboard, SQL results and workbook
- GitHub Actions workflow runs the rebuild and checks.py on every push
- workbook Scenario tab: conservative case and per-1% rows (charts kept)
- README: remove unconfirmed "take-out and delivery" wording, explain the calculated overhead line

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_015ugECwNZWjJ9KEvhL54xSU
</commit_message>
<xml_diff>
--- a/data/Canadian_Restaurant_Benchmark.xlsx
+++ b/data/Canadian_Restaurant_Benchmark.xlsx
@@ -3229,7 +3229,7 @@
     <tabColor rgb="FFE36414"/>
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D37"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="62"/>
@@ -3436,6 +3436,117 @@
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="22" t="s">
         <v>112</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="13" t="inlineStr">
+        <is>
+          <t>Conservative case: overhead cut on the published utilities line only</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>Overhead reduction, utilities and telecom only</t>
+        </is>
+      </c>
+      <c r="B28" s="17" t="n">
+        <f aca="false">B6</f>
+        <v>0.15</v>
+      </c>
+      <c r="C28" s="27" t="n">
+        <f aca="false">Benchmark!B9*B28</f>
+        <v>3225</v>
+      </c>
+      <c r="D28" s="15" t="inlineStr">
+        <is>
+          <t>Utilities x cut. Leaves out the calculated other expenses line.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="25" t="inlineStr">
+        <is>
+          <t>Total profit improvement (conservative)</t>
+        </is>
+      </c>
+      <c r="C29" s="27" t="n">
+        <f aca="false">C5+C28+C8</f>
+        <v>27049</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="15" t="inlineStr">
+        <is>
+          <t>Profit after (conservative)</t>
+        </is>
+      </c>
+      <c r="C30" s="27" t="n">
+        <f aca="false">C11+C29</f>
+        <v>48549</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="15" t="inlineStr">
+        <is>
+          <t>Margin after (conservative)</t>
+        </is>
+      </c>
+      <c r="C31" s="17" t="n">
+        <f aca="false">C30/Benchmark!B5</f>
+        <v>0.05717027790861988</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>Part of the headline overhead gain that comes from the calculated other expenses line</t>
+        </is>
+      </c>
+      <c r="C32" s="27" t="n">
+        <f aca="false">Benchmark!B11*B6</f>
+        <v>19620</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="inlineStr">
+        <is>
+          <t>Profit gain from a 1% cut in each cost line</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="15" t="inlineStr">
+        <is>
+          <t>Cost of sales</t>
+        </is>
+      </c>
+      <c r="C35" s="27" t="n">
+        <f aca="false">Benchmark!B6*0.01</f>
+        <v>3804</v>
+      </c>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="15" t="inlineStr">
+        <is>
+          <t>Labour</t>
+        </is>
+      </c>
+      <c r="C36" s="27" t="n">
+        <f aca="false">Benchmark!B7*0.01</f>
+        <v>2002</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="15" t="inlineStr">
+        <is>
+          <t>Overhead (utilities + calculated other)</t>
+        </is>
+      </c>
+      <c r="C37" s="27" t="n">
+        <f aca="false">(Benchmark!B9+Benchmark!B11)*0.01</f>
+        <v>1523</v>
       </c>
     </row>
   </sheetData>

</xml_diff>